<commit_message>
update algorithm and topology
</commit_message>
<xml_diff>
--- a/temp/definition of rings.xlsx
+++ b/temp/definition of rings.xlsx
@@ -160,20 +160,27 @@
     <t>если нет схождения в кольцо - текущую строку удалить</t>
   </si>
   <si>
-    <t>в конце удалить с конца повторяющиеся линки</t>
-  </si>
-  <si>
     <t>если нет схождения в кольцо - новые строки удалить</t>
+  </si>
+  <si>
+    <t>в конце обхода удалить с конца повторяющиеся линки</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B0F0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -199,9 +206,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -786,12 +794,12 @@
     </row>
     <row r="17" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="18" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B18" s="2" t="s">
         <v>48</v>
-      </c>
-    </row>
-    <row r="18" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="B18" s="1" t="s">
-        <v>49</v>
       </c>
       <c r="I18" s="1" t="s">
         <v>0</v>
@@ -1144,7 +1152,7 @@
       </c>
     </row>
     <row r="31" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="I31" s="1" t="s">
+      <c r="I31" s="2" t="s">
         <v>47</v>
       </c>
     </row>

</xml_diff>